<commit_message>
Add confusion matrix image for T5 model
</commit_message>
<xml_diff>
--- a/datasets/metricas.xlsx
+++ b/datasets/metricas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,13 +452,18 @@
           <t>Precisao</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Rede</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -474,6 +479,11 @@
       </c>
       <c r="G2" t="n">
         <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -481,7 +491,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -497,6 +507,11 @@
       </c>
       <c r="G3" t="n">
         <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -504,7 +519,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -520,6 +535,11 @@
       </c>
       <c r="G4" t="n">
         <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -527,7 +547,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -543,6 +563,11 @@
       </c>
       <c r="G5" t="n">
         <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -550,7 +575,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -566,6 +591,11 @@
       </c>
       <c r="G6" t="n">
         <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update main branch with recent changes Incorporate the latest updates and improvements to the main branch, enhancing overall functionality and performance.
</commit_message>
<xml_diff>
--- a/datasets/metricas.xlsx
+++ b/datasets/metricas.xlsx
@@ -413,189 +413,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>MODELOS</t>
+          <t>Rede</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Acertos</t>
+          <t>Erro relativo medio (%)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Erros</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Acurácia</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Sensibilidade</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Especificidade</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Precisao</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Rede</t>
+          <t>Variancia (%)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>18</v>
+        <v>2.3309</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
+        <v>3.3043</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>1.7742</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
+        <v>1.9988</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>1.3758</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
+        <v>1.4982</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>2.8337</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
+        <v>3.8368</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>1.3391</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
+        <v>1.1864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza arquivos de métricas e gráficos de validação com novos dados
</commit_message>
<xml_diff>
--- a/datasets/metricas.xlsx
+++ b/datasets/metricas.xlsx
@@ -440,10 +440,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.3309</v>
+        <v>1.2184</v>
       </c>
       <c r="C2" t="n">
-        <v>3.3043</v>
+        <v>1.0152</v>
       </c>
     </row>
     <row r="3">
@@ -453,10 +453,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.7742</v>
+        <v>1.2301</v>
       </c>
       <c r="C3" t="n">
-        <v>1.9988</v>
+        <v>1.5967</v>
       </c>
     </row>
     <row r="4">
@@ -466,10 +466,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.3758</v>
+        <v>1.5815</v>
       </c>
       <c r="C4" t="n">
-        <v>1.4982</v>
+        <v>1.8049</v>
       </c>
     </row>
     <row r="5">
@@ -479,10 +479,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.8337</v>
+        <v>1.9322</v>
       </c>
       <c r="C5" t="n">
-        <v>3.8368</v>
+        <v>1.5992</v>
       </c>
     </row>
     <row r="6">
@@ -492,10 +492,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.3391</v>
+        <v>2.0084</v>
       </c>
       <c r="C6" t="n">
-        <v>1.1864</v>
+        <v>3.8394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>